<commit_message>
Comprehensive update: 0521-0604 data pipeline + 06 DataMining tools
- 01: 竞价空间分析(预测/实际) 0517-0604, including new forecast templates
- 02: 日前机组组合收益复盘 0526-0601
- 03: 实时机组组合收益复盘 0525-0531
- 04: 日结算收益复盘 0522-0524, settlement statements
- 05: 统计表更新(日前+实时+日结算), incremental update support
- 06: db_viewer, extract_prices, intraday_viz, generate_analysis_html (bidding+price+weather), reserve capacity analysis, peak-valley analysis
- Docs: CLAUDE.md expanded with DB schema, 天机数据库 table index, 电价分析手册, 策略复盘结论
</commit_message>
<xml_diff>
--- a/01 biddingSpace_analysis/assets/输出模版-0521-竞价空间分析.xlsx
+++ b/01 biddingSpace_analysis/assets/输出模版-0521-竞价空间分析.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\百度网盘同步空间\01 电力交易与储能\01 各省项目及政策\04山东\每日策略实例\2026\05月\0518-阴雨\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\DataWork\Storage_Strategy\01 biddingSpace_analysis\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61AE66D1-9D93-4281-A7EB-BAE470D2033C}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2336764-FB5A-49E6-BDEF-7C9BB2D77AE6}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12648" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="786" uniqueCount="452">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="786" uniqueCount="455">
   <si>
     <t>时刻</t>
   </si>
@@ -328,9 +328,6 @@
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
-    <t>预测</t>
-  </si>
-  <si>
     <t>竞价最小值</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
@@ -1392,6 +1389,22 @@
   </si>
   <si>
     <t>0.79</t>
+  </si>
+  <si>
+    <t>直调负荷</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>联络线受电负荷</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>风电总加</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>光伏总加</t>
+    <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -7381,1174 +7394,1174 @@
     </row>
     <row r="3" spans="1:97" ht="27.6" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>99</v>
+        <v>451</v>
       </c>
       <c r="B3" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="C3" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="D3" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="E3" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="F3" s="2" t="s">
         <v>114</v>
       </c>
-      <c r="F3" s="2" t="s">
+      <c r="G3" s="2" t="s">
         <v>115</v>
       </c>
-      <c r="G3" s="2" t="s">
+      <c r="H3" s="2" t="s">
         <v>116</v>
       </c>
-      <c r="H3" s="2" t="s">
+      <c r="I3" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="I3" s="2" t="s">
+      <c r="J3" s="2" t="s">
         <v>118</v>
       </c>
-      <c r="J3" s="2" t="s">
+      <c r="K3" s="2" t="s">
         <v>119</v>
       </c>
-      <c r="K3" s="2" t="s">
+      <c r="L3" s="2" t="s">
         <v>120</v>
       </c>
-      <c r="L3" s="2" t="s">
+      <c r="M3" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="N3" s="2" t="s">
         <v>121</v>
       </c>
-      <c r="M3" s="2" t="s">
-        <v>121</v>
-      </c>
-      <c r="N3" s="2" t="s">
+      <c r="O3" s="2" t="s">
         <v>122</v>
       </c>
-      <c r="O3" s="2" t="s">
+      <c r="P3" s="2" t="s">
         <v>123</v>
       </c>
-      <c r="P3" s="2" t="s">
+      <c r="Q3" s="2" t="s">
         <v>124</v>
       </c>
-      <c r="Q3" s="2" t="s">
+      <c r="R3" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="S3" s="2" t="s">
         <v>125</v>
       </c>
-      <c r="R3" s="2" t="s">
-        <v>120</v>
-      </c>
-      <c r="S3" s="2" t="s">
+      <c r="T3" s="2" t="s">
         <v>126</v>
       </c>
-      <c r="T3" s="2" t="s">
+      <c r="U3" s="2" t="s">
         <v>127</v>
       </c>
-      <c r="U3" s="2" t="s">
+      <c r="V3" s="2" t="s">
         <v>128</v>
       </c>
-      <c r="V3" s="2" t="s">
+      <c r="W3" s="2" t="s">
         <v>129</v>
       </c>
-      <c r="W3" s="2" t="s">
+      <c r="X3" s="2" t="s">
         <v>130</v>
       </c>
-      <c r="X3" s="2" t="s">
+      <c r="Y3" s="2" t="s">
         <v>131</v>
       </c>
-      <c r="Y3" s="2" t="s">
+      <c r="Z3" s="2" t="s">
         <v>132</v>
       </c>
-      <c r="Z3" s="2" t="s">
+      <c r="AA3" s="2" t="s">
         <v>133</v>
       </c>
-      <c r="AA3" s="2" t="s">
+      <c r="AB3" s="2" t="s">
         <v>134</v>
       </c>
-      <c r="AB3" s="2" t="s">
+      <c r="AC3" s="2" t="s">
         <v>135</v>
       </c>
-      <c r="AC3" s="2" t="s">
+      <c r="AD3" s="2" t="s">
         <v>136</v>
       </c>
-      <c r="AD3" s="2" t="s">
+      <c r="AE3" s="2" t="s">
         <v>137</v>
       </c>
-      <c r="AE3" s="2" t="s">
+      <c r="AF3" s="2" t="s">
         <v>138</v>
       </c>
-      <c r="AF3" s="2" t="s">
+      <c r="AG3" s="2" t="s">
         <v>139</v>
       </c>
-      <c r="AG3" s="2" t="s">
+      <c r="AH3" s="2" t="s">
         <v>140</v>
       </c>
-      <c r="AH3" s="2" t="s">
+      <c r="AI3" s="2" t="s">
         <v>141</v>
       </c>
-      <c r="AI3" s="2" t="s">
+      <c r="AJ3" s="2" t="s">
         <v>142</v>
       </c>
-      <c r="AJ3" s="2" t="s">
+      <c r="AK3" s="2" t="s">
         <v>143</v>
       </c>
-      <c r="AK3" s="2" t="s">
+      <c r="AL3" s="2" t="s">
         <v>144</v>
       </c>
-      <c r="AL3" s="2" t="s">
+      <c r="AM3" s="2" t="s">
         <v>145</v>
       </c>
-      <c r="AM3" s="2" t="s">
+      <c r="AN3" s="2" t="s">
         <v>146</v>
       </c>
-      <c r="AN3" s="2" t="s">
+      <c r="AO3" s="2" t="s">
         <v>147</v>
       </c>
-      <c r="AO3" s="2" t="s">
+      <c r="AP3" s="2" t="s">
         <v>148</v>
       </c>
-      <c r="AP3" s="2" t="s">
+      <c r="AQ3" s="2" t="s">
         <v>149</v>
       </c>
-      <c r="AQ3" s="2" t="s">
+      <c r="AR3" s="2" t="s">
         <v>150</v>
       </c>
-      <c r="AR3" s="2" t="s">
+      <c r="AS3" s="2" t="s">
         <v>151</v>
       </c>
-      <c r="AS3" s="2" t="s">
+      <c r="AT3" s="2" t="s">
         <v>152</v>
       </c>
-      <c r="AT3" s="2" t="s">
+      <c r="AU3" s="2" t="s">
         <v>153</v>
       </c>
-      <c r="AU3" s="2" t="s">
+      <c r="AV3" s="2" t="s">
         <v>154</v>
       </c>
-      <c r="AV3" s="2" t="s">
+      <c r="AW3" s="2" t="s">
         <v>155</v>
       </c>
-      <c r="AW3" s="2" t="s">
+      <c r="AX3" s="2" t="s">
         <v>156</v>
       </c>
-      <c r="AX3" s="2" t="s">
+      <c r="AY3" s="2" t="s">
         <v>157</v>
       </c>
-      <c r="AY3" s="2" t="s">
+      <c r="AZ3" s="2" t="s">
         <v>158</v>
       </c>
-      <c r="AZ3" s="2" t="s">
+      <c r="BA3" s="2" t="s">
         <v>159</v>
       </c>
-      <c r="BA3" s="2" t="s">
+      <c r="BB3" s="2" t="s">
         <v>160</v>
       </c>
-      <c r="BB3" s="2" t="s">
+      <c r="BC3" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="BC3" s="2" t="s">
+      <c r="BD3" s="2" t="s">
         <v>162</v>
       </c>
-      <c r="BD3" s="2" t="s">
+      <c r="BE3" s="2" t="s">
         <v>163</v>
       </c>
-      <c r="BE3" s="2" t="s">
+      <c r="BF3" s="2" t="s">
         <v>164</v>
       </c>
-      <c r="BF3" s="2" t="s">
+      <c r="BG3" s="2" t="s">
         <v>165</v>
       </c>
-      <c r="BG3" s="2" t="s">
+      <c r="BH3" s="2" t="s">
         <v>166</v>
       </c>
-      <c r="BH3" s="2" t="s">
+      <c r="BI3" s="2" t="s">
         <v>167</v>
       </c>
-      <c r="BI3" s="2" t="s">
+      <c r="BJ3" s="2" t="s">
         <v>168</v>
       </c>
-      <c r="BJ3" s="2" t="s">
+      <c r="BK3" s="2" t="s">
         <v>169</v>
       </c>
-      <c r="BK3" s="2" t="s">
+      <c r="BL3" s="2" t="s">
         <v>170</v>
       </c>
-      <c r="BL3" s="2" t="s">
+      <c r="BM3" s="2" t="s">
         <v>171</v>
       </c>
-      <c r="BM3" s="2" t="s">
+      <c r="BN3" s="2" t="s">
         <v>172</v>
       </c>
-      <c r="BN3" s="2" t="s">
+      <c r="BO3" s="2" t="s">
         <v>173</v>
       </c>
-      <c r="BO3" s="2" t="s">
+      <c r="BP3" s="2" t="s">
         <v>174</v>
       </c>
-      <c r="BP3" s="2" t="s">
+      <c r="BQ3" s="2" t="s">
         <v>175</v>
       </c>
-      <c r="BQ3" s="2" t="s">
+      <c r="BR3" s="2" t="s">
         <v>176</v>
       </c>
-      <c r="BR3" s="2" t="s">
+      <c r="BS3" s="2" t="s">
         <v>177</v>
       </c>
-      <c r="BS3" s="2" t="s">
+      <c r="BT3" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="BT3" s="2" t="s">
+      <c r="BU3" s="2" t="s">
         <v>179</v>
       </c>
-      <c r="BU3" s="2" t="s">
+      <c r="BV3" s="2" t="s">
         <v>180</v>
       </c>
-      <c r="BV3" s="2" t="s">
+      <c r="BW3" s="2" t="s">
         <v>181</v>
       </c>
-      <c r="BW3" s="2" t="s">
+      <c r="BX3" s="2" t="s">
         <v>182</v>
       </c>
-      <c r="BX3" s="2" t="s">
+      <c r="BY3" s="2" t="s">
         <v>183</v>
       </c>
-      <c r="BY3" s="2" t="s">
+      <c r="BZ3" s="2" t="s">
         <v>184</v>
       </c>
-      <c r="BZ3" s="2" t="s">
+      <c r="CA3" s="2" t="s">
         <v>185</v>
       </c>
-      <c r="CA3" s="2" t="s">
+      <c r="CB3" s="2" t="s">
         <v>186</v>
       </c>
-      <c r="CB3" s="2" t="s">
+      <c r="CC3" s="2" t="s">
         <v>187</v>
       </c>
-      <c r="CC3" s="2" t="s">
+      <c r="CD3" s="2" t="s">
         <v>188</v>
       </c>
-      <c r="CD3" s="2" t="s">
+      <c r="CE3" s="2" t="s">
         <v>189</v>
       </c>
-      <c r="CE3" s="2" t="s">
+      <c r="CF3" s="2" t="s">
         <v>190</v>
       </c>
-      <c r="CF3" s="2" t="s">
+      <c r="CG3" s="2" t="s">
         <v>191</v>
       </c>
-      <c r="CG3" s="2" t="s">
+      <c r="CH3" s="2" t="s">
         <v>192</v>
       </c>
-      <c r="CH3" s="2" t="s">
+      <c r="CI3" s="2" t="s">
         <v>193</v>
       </c>
-      <c r="CI3" s="2" t="s">
+      <c r="CJ3" s="2" t="s">
         <v>194</v>
       </c>
-      <c r="CJ3" s="2" t="s">
+      <c r="CK3" s="2" t="s">
         <v>195</v>
       </c>
-      <c r="CK3" s="2" t="s">
+      <c r="CL3" s="2" t="s">
         <v>196</v>
       </c>
-      <c r="CL3" s="2" t="s">
+      <c r="CM3" s="2" t="s">
         <v>197</v>
       </c>
-      <c r="CM3" s="2" t="s">
+      <c r="CN3" s="2" t="s">
         <v>198</v>
       </c>
-      <c r="CN3" s="2" t="s">
+      <c r="CO3" s="2" t="s">
         <v>199</v>
       </c>
-      <c r="CO3" s="2" t="s">
+      <c r="CP3" s="2" t="s">
         <v>200</v>
       </c>
-      <c r="CP3" s="2" t="s">
+      <c r="CQ3" s="2" t="s">
         <v>201</v>
       </c>
-      <c r="CQ3" s="2" t="s">
+      <c r="CR3" s="2" t="s">
         <v>202</v>
       </c>
-      <c r="CR3" s="2" t="s">
+      <c r="CS3" s="2" t="s">
         <v>203</v>
-      </c>
-      <c r="CS3" s="2" t="s">
-        <v>204</v>
       </c>
     </row>
     <row r="4" spans="1:97" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>99</v>
+        <v>452</v>
       </c>
       <c r="B4" s="2" t="s">
+        <v>204</v>
+      </c>
+      <c r="C4" s="2" t="s">
         <v>205</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="D4" s="2" t="s">
         <v>206</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="E4" s="2" t="s">
         <v>207</v>
       </c>
-      <c r="E4" s="2" t="s">
+      <c r="F4" s="2" t="s">
         <v>208</v>
       </c>
-      <c r="F4" s="2" t="s">
+      <c r="G4" s="2" t="s">
         <v>209</v>
       </c>
-      <c r="G4" s="2" t="s">
+      <c r="H4" s="2" t="s">
         <v>210</v>
       </c>
-      <c r="H4" s="2" t="s">
+      <c r="I4" s="2" t="s">
         <v>211</v>
       </c>
-      <c r="I4" s="2" t="s">
+      <c r="J4" s="2" t="s">
         <v>212</v>
       </c>
-      <c r="J4" s="2" t="s">
+      <c r="K4" s="2" t="s">
         <v>213</v>
       </c>
-      <c r="K4" s="2" t="s">
+      <c r="L4" s="2" t="s">
         <v>214</v>
       </c>
-      <c r="L4" s="2" t="s">
+      <c r="M4" s="2" t="s">
         <v>215</v>
       </c>
-      <c r="M4" s="2" t="s">
+      <c r="N4" s="2" t="s">
+        <v>215</v>
+      </c>
+      <c r="O4" s="2" t="s">
         <v>216</v>
       </c>
-      <c r="N4" s="2" t="s">
-        <v>216</v>
-      </c>
-      <c r="O4" s="2" t="s">
+      <c r="P4" s="2" t="s">
         <v>217</v>
       </c>
-      <c r="P4" s="2" t="s">
+      <c r="Q4" s="2" t="s">
         <v>218</v>
       </c>
-      <c r="Q4" s="2" t="s">
+      <c r="R4" s="2" t="s">
         <v>219</v>
       </c>
-      <c r="R4" s="2" t="s">
+      <c r="S4" s="2" t="s">
         <v>220</v>
       </c>
-      <c r="S4" s="2" t="s">
+      <c r="T4" s="2" t="s">
         <v>221</v>
       </c>
-      <c r="T4" s="2" t="s">
+      <c r="U4" s="2" t="s">
         <v>222</v>
       </c>
-      <c r="U4" s="2" t="s">
+      <c r="V4" s="2" t="s">
         <v>223</v>
       </c>
-      <c r="V4" s="2" t="s">
+      <c r="W4" s="2" t="s">
         <v>224</v>
       </c>
-      <c r="W4" s="2" t="s">
+      <c r="X4" s="2" t="s">
         <v>225</v>
       </c>
-      <c r="X4" s="2" t="s">
+      <c r="Y4" s="2" t="s">
         <v>226</v>
       </c>
-      <c r="Y4" s="2" t="s">
+      <c r="Z4" s="2" t="s">
         <v>227</v>
       </c>
-      <c r="Z4" s="2" t="s">
+      <c r="AA4" s="2" t="s">
         <v>228</v>
       </c>
-      <c r="AA4" s="2" t="s">
+      <c r="AB4" s="2" t="s">
         <v>229</v>
       </c>
-      <c r="AB4" s="2" t="s">
+      <c r="AC4" s="2" t="s">
         <v>230</v>
       </c>
-      <c r="AC4" s="2" t="s">
+      <c r="AD4" s="2" t="s">
         <v>231</v>
       </c>
-      <c r="AD4" s="2" t="s">
+      <c r="AE4" s="2" t="s">
         <v>232</v>
       </c>
-      <c r="AE4" s="2" t="s">
+      <c r="AF4" s="2" t="s">
         <v>233</v>
       </c>
-      <c r="AF4" s="2" t="s">
+      <c r="AG4" s="2" t="s">
         <v>234</v>
       </c>
-      <c r="AG4" s="2" t="s">
+      <c r="AH4" s="2" t="s">
         <v>235</v>
       </c>
-      <c r="AH4" s="2" t="s">
+      <c r="AI4" s="2" t="s">
         <v>236</v>
       </c>
-      <c r="AI4" s="2" t="s">
+      <c r="AJ4" s="2" t="s">
         <v>237</v>
       </c>
-      <c r="AJ4" s="2" t="s">
+      <c r="AK4" s="2" t="s">
         <v>238</v>
       </c>
-      <c r="AK4" s="2" t="s">
+      <c r="AL4" s="2" t="s">
         <v>239</v>
       </c>
-      <c r="AL4" s="2" t="s">
+      <c r="AM4" s="2" t="s">
         <v>240</v>
       </c>
-      <c r="AM4" s="2" t="s">
+      <c r="AN4" s="2" t="s">
         <v>241</v>
       </c>
-      <c r="AN4" s="2" t="s">
+      <c r="AO4" s="2" t="s">
         <v>242</v>
       </c>
-      <c r="AO4" s="2" t="s">
+      <c r="AP4" s="2" t="s">
         <v>243</v>
       </c>
-      <c r="AP4" s="2" t="s">
+      <c r="AQ4" s="2" t="s">
         <v>244</v>
       </c>
-      <c r="AQ4" s="2" t="s">
+      <c r="AR4" s="2" t="s">
         <v>245</v>
       </c>
-      <c r="AR4" s="2" t="s">
+      <c r="AS4" s="2" t="s">
         <v>246</v>
       </c>
-      <c r="AS4" s="2" t="s">
+      <c r="AT4" s="2" t="s">
         <v>247</v>
       </c>
-      <c r="AT4" s="2" t="s">
+      <c r="AU4" s="2" t="s">
+        <v>247</v>
+      </c>
+      <c r="AV4" s="2" t="s">
+        <v>247</v>
+      </c>
+      <c r="AW4" s="2" t="s">
+        <v>247</v>
+      </c>
+      <c r="AX4" s="2" t="s">
+        <v>247</v>
+      </c>
+      <c r="AY4" s="2" t="s">
         <v>248</v>
       </c>
-      <c r="AU4" s="2" t="s">
-        <v>248</v>
-      </c>
-      <c r="AV4" s="2" t="s">
-        <v>248</v>
-      </c>
-      <c r="AW4" s="2" t="s">
-        <v>248</v>
-      </c>
-      <c r="AX4" s="2" t="s">
-        <v>248</v>
-      </c>
-      <c r="AY4" s="2" t="s">
+      <c r="AZ4" s="2" t="s">
         <v>249</v>
       </c>
-      <c r="AZ4" s="2" t="s">
+      <c r="BA4" s="2" t="s">
         <v>250</v>
       </c>
-      <c r="BA4" s="2" t="s">
+      <c r="BB4" s="2" t="s">
         <v>251</v>
       </c>
-      <c r="BB4" s="2" t="s">
+      <c r="BC4" s="2" t="s">
         <v>252</v>
       </c>
-      <c r="BC4" s="2" t="s">
+      <c r="BD4" s="2" t="s">
         <v>253</v>
       </c>
-      <c r="BD4" s="2" t="s">
+      <c r="BE4" s="2" t="s">
         <v>254</v>
       </c>
-      <c r="BE4" s="2" t="s">
+      <c r="BF4" s="2" t="s">
         <v>255</v>
       </c>
-      <c r="BF4" s="2" t="s">
+      <c r="BG4" s="2" t="s">
         <v>256</v>
       </c>
-      <c r="BG4" s="2" t="s">
+      <c r="BH4" s="2" t="s">
         <v>257</v>
       </c>
-      <c r="BH4" s="2" t="s">
+      <c r="BI4" s="2" t="s">
         <v>258</v>
       </c>
-      <c r="BI4" s="2" t="s">
+      <c r="BJ4" s="2" t="s">
         <v>259</v>
       </c>
-      <c r="BJ4" s="2" t="s">
+      <c r="BK4" s="2" t="s">
         <v>260</v>
       </c>
-      <c r="BK4" s="2" t="s">
+      <c r="BL4" s="2" t="s">
         <v>261</v>
       </c>
-      <c r="BL4" s="2" t="s">
+      <c r="BM4" s="2" t="s">
         <v>262</v>
       </c>
-      <c r="BM4" s="2" t="s">
+      <c r="BN4" s="2" t="s">
         <v>263</v>
       </c>
-      <c r="BN4" s="2" t="s">
+      <c r="BO4" s="2" t="s">
         <v>264</v>
       </c>
-      <c r="BO4" s="2" t="s">
+      <c r="BP4" s="2" t="s">
         <v>265</v>
       </c>
-      <c r="BP4" s="2" t="s">
+      <c r="BQ4" s="2" t="s">
         <v>266</v>
       </c>
-      <c r="BQ4" s="2" t="s">
+      <c r="BR4" s="2" t="s">
         <v>267</v>
       </c>
-      <c r="BR4" s="2" t="s">
+      <c r="BS4" s="2" t="s">
         <v>268</v>
       </c>
-      <c r="BS4" s="2" t="s">
+      <c r="BT4" s="2" t="s">
+        <v>268</v>
+      </c>
+      <c r="BU4" s="2" t="s">
         <v>269</v>
       </c>
-      <c r="BT4" s="2" t="s">
-        <v>269</v>
-      </c>
-      <c r="BU4" s="2" t="s">
+      <c r="BV4" s="2" t="s">
         <v>270</v>
       </c>
-      <c r="BV4" s="2" t="s">
+      <c r="BW4" s="2" t="s">
         <v>271</v>
       </c>
-      <c r="BW4" s="2" t="s">
+      <c r="BX4" s="2" t="s">
         <v>272</v>
       </c>
-      <c r="BX4" s="2" t="s">
+      <c r="BY4" s="2" t="s">
         <v>273</v>
       </c>
-      <c r="BY4" s="2" t="s">
+      <c r="BZ4" s="2" t="s">
         <v>274</v>
       </c>
-      <c r="BZ4" s="2" t="s">
+      <c r="CA4" s="2" t="s">
         <v>275</v>
       </c>
-      <c r="CA4" s="2" t="s">
+      <c r="CB4" s="2" t="s">
         <v>276</v>
       </c>
-      <c r="CB4" s="2" t="s">
+      <c r="CC4" s="2" t="s">
         <v>277</v>
       </c>
-      <c r="CC4" s="2" t="s">
+      <c r="CD4" s="2" t="s">
         <v>278</v>
       </c>
-      <c r="CD4" s="2" t="s">
+      <c r="CE4" s="2" t="s">
         <v>279</v>
       </c>
-      <c r="CE4" s="2" t="s">
+      <c r="CF4" s="2" t="s">
         <v>280</v>
       </c>
-      <c r="CF4" s="2" t="s">
+      <c r="CG4" s="2" t="s">
         <v>281</v>
       </c>
-      <c r="CG4" s="2" t="s">
+      <c r="CH4" s="2" t="s">
         <v>282</v>
       </c>
-      <c r="CH4" s="2" t="s">
+      <c r="CI4" s="2" t="s">
         <v>283</v>
       </c>
-      <c r="CI4" s="2" t="s">
+      <c r="CJ4" s="2" t="s">
         <v>284</v>
       </c>
-      <c r="CJ4" s="2" t="s">
+      <c r="CK4" s="2" t="s">
         <v>285</v>
       </c>
-      <c r="CK4" s="2" t="s">
+      <c r="CL4" s="2" t="s">
         <v>286</v>
       </c>
-      <c r="CL4" s="2" t="s">
+      <c r="CM4" s="2" t="s">
         <v>287</v>
       </c>
-      <c r="CM4" s="2" t="s">
+      <c r="CN4" s="2" t="s">
         <v>288</v>
       </c>
-      <c r="CN4" s="2" t="s">
+      <c r="CO4" s="2" t="s">
         <v>289</v>
       </c>
-      <c r="CO4" s="2" t="s">
+      <c r="CP4" s="2" t="s">
         <v>290</v>
       </c>
-      <c r="CP4" s="2" t="s">
+      <c r="CQ4" s="2" t="s">
         <v>291</v>
       </c>
-      <c r="CQ4" s="2" t="s">
+      <c r="CR4" s="2" t="s">
         <v>292</v>
       </c>
-      <c r="CR4" s="2" t="s">
+      <c r="CS4" s="2" t="s">
         <v>293</v>
-      </c>
-      <c r="CS4" s="2" t="s">
-        <v>294</v>
       </c>
     </row>
     <row r="5" spans="1:97" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>99</v>
+        <v>453</v>
       </c>
       <c r="B5" s="2" t="s">
+        <v>294</v>
+      </c>
+      <c r="C5" s="2" t="s">
         <v>295</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="D5" s="2" t="s">
         <v>296</v>
       </c>
-      <c r="D5" s="2" t="s">
+      <c r="E5" s="2" t="s">
         <v>297</v>
       </c>
-      <c r="E5" s="2" t="s">
+      <c r="F5" s="2" t="s">
         <v>298</v>
       </c>
-      <c r="F5" s="2" t="s">
+      <c r="G5" s="2" t="s">
         <v>299</v>
       </c>
-      <c r="G5" s="2" t="s">
+      <c r="H5" s="2" t="s">
         <v>300</v>
       </c>
-      <c r="H5" s="2" t="s">
+      <c r="I5" s="2" t="s">
         <v>301</v>
       </c>
-      <c r="I5" s="2" t="s">
+      <c r="J5" s="2" t="s">
         <v>302</v>
       </c>
-      <c r="J5" s="2" t="s">
+      <c r="K5" s="2" t="s">
         <v>303</v>
       </c>
-      <c r="K5" s="2" t="s">
+      <c r="L5" s="2" t="s">
         <v>304</v>
       </c>
-      <c r="L5" s="2" t="s">
+      <c r="M5" s="2" t="s">
         <v>305</v>
       </c>
-      <c r="M5" s="2" t="s">
+      <c r="N5" s="2" t="s">
         <v>306</v>
       </c>
-      <c r="N5" s="2" t="s">
+      <c r="O5" s="2" t="s">
         <v>307</v>
       </c>
-      <c r="O5" s="2" t="s">
+      <c r="P5" s="2" t="s">
         <v>308</v>
       </c>
-      <c r="P5" s="2" t="s">
+      <c r="Q5" s="2" t="s">
         <v>309</v>
       </c>
-      <c r="Q5" s="2" t="s">
+      <c r="R5" s="2" t="s">
         <v>310</v>
       </c>
-      <c r="R5" s="2" t="s">
+      <c r="S5" s="2" t="s">
         <v>311</v>
       </c>
-      <c r="S5" s="2" t="s">
+      <c r="T5" s="2" t="s">
         <v>312</v>
       </c>
-      <c r="T5" s="2" t="s">
+      <c r="U5" s="2" t="s">
         <v>313</v>
       </c>
-      <c r="U5" s="2" t="s">
+      <c r="V5" s="2" t="s">
         <v>314</v>
       </c>
-      <c r="V5" s="2" t="s">
+      <c r="W5" s="2" t="s">
         <v>315</v>
       </c>
-      <c r="W5" s="2" t="s">
+      <c r="X5" s="2" t="s">
         <v>316</v>
       </c>
-      <c r="X5" s="2" t="s">
+      <c r="Y5" s="2" t="s">
         <v>317</v>
       </c>
-      <c r="Y5" s="2" t="s">
+      <c r="Z5" s="2" t="s">
         <v>318</v>
       </c>
-      <c r="Z5" s="2" t="s">
+      <c r="AA5" s="2" t="s">
         <v>319</v>
       </c>
-      <c r="AA5" s="2" t="s">
+      <c r="AB5" s="2" t="s">
         <v>320</v>
       </c>
-      <c r="AB5" s="2" t="s">
+      <c r="AC5" s="2" t="s">
         <v>321</v>
       </c>
-      <c r="AC5" s="2" t="s">
+      <c r="AD5" s="2" t="s">
         <v>322</v>
       </c>
-      <c r="AD5" s="2" t="s">
+      <c r="AE5" s="2" t="s">
         <v>323</v>
       </c>
-      <c r="AE5" s="2" t="s">
+      <c r="AF5" s="2" t="s">
         <v>324</v>
       </c>
-      <c r="AF5" s="2" t="s">
+      <c r="AG5" s="2" t="s">
         <v>325</v>
       </c>
-      <c r="AG5" s="2" t="s">
+      <c r="AH5" s="2" t="s">
         <v>326</v>
       </c>
-      <c r="AH5" s="2" t="s">
+      <c r="AI5" s="2" t="s">
         <v>327</v>
       </c>
-      <c r="AI5" s="2" t="s">
+      <c r="AJ5" s="2" t="s">
         <v>328</v>
       </c>
-      <c r="AJ5" s="2" t="s">
+      <c r="AK5" s="2" t="s">
         <v>329</v>
       </c>
-      <c r="AK5" s="2" t="s">
+      <c r="AL5" s="2" t="s">
         <v>330</v>
       </c>
-      <c r="AL5" s="2" t="s">
+      <c r="AM5" s="2" t="s">
         <v>331</v>
       </c>
-      <c r="AM5" s="2" t="s">
+      <c r="AN5" s="2" t="s">
         <v>332</v>
       </c>
-      <c r="AN5" s="2" t="s">
+      <c r="AO5" s="2" t="s">
         <v>333</v>
       </c>
-      <c r="AO5" s="2" t="s">
+      <c r="AP5" s="2" t="s">
         <v>334</v>
       </c>
-      <c r="AP5" s="2" t="s">
+      <c r="AQ5" s="2" t="s">
         <v>335</v>
       </c>
-      <c r="AQ5" s="2" t="s">
+      <c r="AR5" s="2" t="s">
         <v>336</v>
       </c>
-      <c r="AR5" s="2" t="s">
+      <c r="AS5" s="2" t="s">
         <v>337</v>
       </c>
-      <c r="AS5" s="2" t="s">
+      <c r="AT5" s="2" t="s">
         <v>338</v>
       </c>
-      <c r="AT5" s="2" t="s">
+      <c r="AU5" s="2" t="s">
         <v>339</v>
       </c>
-      <c r="AU5" s="2" t="s">
+      <c r="AV5" s="2" t="s">
         <v>340</v>
       </c>
-      <c r="AV5" s="2" t="s">
+      <c r="AW5" s="2" t="s">
         <v>341</v>
       </c>
-      <c r="AW5" s="2" t="s">
+      <c r="AX5" s="2" t="s">
         <v>342</v>
       </c>
-      <c r="AX5" s="2" t="s">
+      <c r="AY5" s="2" t="s">
         <v>343</v>
       </c>
-      <c r="AY5" s="2" t="s">
+      <c r="AZ5" s="2" t="s">
         <v>344</v>
       </c>
-      <c r="AZ5" s="2" t="s">
+      <c r="BA5" s="2" t="s">
         <v>345</v>
       </c>
-      <c r="BA5" s="2" t="s">
+      <c r="BB5" s="2" t="s">
         <v>346</v>
       </c>
-      <c r="BB5" s="2" t="s">
+      <c r="BC5" s="2" t="s">
         <v>347</v>
       </c>
-      <c r="BC5" s="2" t="s">
+      <c r="BD5" s="2" t="s">
         <v>348</v>
       </c>
-      <c r="BD5" s="2" t="s">
+      <c r="BE5" s="2" t="s">
         <v>349</v>
       </c>
-      <c r="BE5" s="2" t="s">
+      <c r="BF5" s="2" t="s">
         <v>350</v>
       </c>
-      <c r="BF5" s="2" t="s">
+      <c r="BG5" s="2" t="s">
         <v>351</v>
       </c>
-      <c r="BG5" s="2" t="s">
+      <c r="BH5" s="2" t="s">
         <v>352</v>
       </c>
-      <c r="BH5" s="2" t="s">
+      <c r="BI5" s="2" t="s">
         <v>353</v>
       </c>
-      <c r="BI5" s="2" t="s">
+      <c r="BJ5" s="2" t="s">
         <v>354</v>
       </c>
-      <c r="BJ5" s="2" t="s">
+      <c r="BK5" s="2" t="s">
         <v>355</v>
       </c>
-      <c r="BK5" s="2" t="s">
+      <c r="BL5" s="2" t="s">
         <v>356</v>
       </c>
-      <c r="BL5" s="2" t="s">
+      <c r="BM5" s="2" t="s">
         <v>357</v>
       </c>
-      <c r="BM5" s="2" t="s">
+      <c r="BN5" s="2" t="s">
         <v>358</v>
       </c>
-      <c r="BN5" s="2" t="s">
+      <c r="BO5" s="2" t="s">
         <v>359</v>
       </c>
-      <c r="BO5" s="2" t="s">
+      <c r="BP5" s="2" t="s">
         <v>360</v>
       </c>
-      <c r="BP5" s="2" t="s">
+      <c r="BQ5" s="2" t="s">
         <v>361</v>
       </c>
-      <c r="BQ5" s="2" t="s">
+      <c r="BR5" s="2" t="s">
         <v>362</v>
       </c>
-      <c r="BR5" s="2" t="s">
+      <c r="BS5" s="2" t="s">
         <v>363</v>
       </c>
-      <c r="BS5" s="2" t="s">
+      <c r="BT5" s="2" t="s">
         <v>364</v>
       </c>
-      <c r="BT5" s="2" t="s">
+      <c r="BU5" s="2" t="s">
         <v>365</v>
       </c>
-      <c r="BU5" s="2" t="s">
+      <c r="BV5" s="2" t="s">
         <v>366</v>
       </c>
-      <c r="BV5" s="2" t="s">
+      <c r="BW5" s="2" t="s">
         <v>367</v>
       </c>
-      <c r="BW5" s="2" t="s">
+      <c r="BX5" s="2" t="s">
         <v>368</v>
       </c>
-      <c r="BX5" s="2" t="s">
+      <c r="BY5" s="2" t="s">
         <v>369</v>
       </c>
-      <c r="BY5" s="2" t="s">
+      <c r="BZ5" s="2" t="s">
         <v>370</v>
       </c>
-      <c r="BZ5" s="2" t="s">
+      <c r="CA5" s="2" t="s">
         <v>371</v>
       </c>
-      <c r="CA5" s="2" t="s">
+      <c r="CB5" s="2" t="s">
         <v>372</v>
       </c>
-      <c r="CB5" s="2" t="s">
+      <c r="CC5" s="2" t="s">
         <v>373</v>
       </c>
-      <c r="CC5" s="2" t="s">
+      <c r="CD5" s="2" t="s">
         <v>374</v>
       </c>
-      <c r="CD5" s="2" t="s">
+      <c r="CE5" s="2" t="s">
         <v>375</v>
       </c>
-      <c r="CE5" s="2" t="s">
+      <c r="CF5" s="2" t="s">
         <v>376</v>
       </c>
-      <c r="CF5" s="2" t="s">
+      <c r="CG5" s="2" t="s">
         <v>377</v>
       </c>
-      <c r="CG5" s="2" t="s">
+      <c r="CH5" s="2" t="s">
         <v>378</v>
       </c>
-      <c r="CH5" s="2" t="s">
+      <c r="CI5" s="2" t="s">
         <v>379</v>
       </c>
-      <c r="CI5" s="2" t="s">
+      <c r="CJ5" s="2" t="s">
         <v>380</v>
       </c>
-      <c r="CJ5" s="2" t="s">
+      <c r="CK5" s="2" t="s">
         <v>381</v>
       </c>
-      <c r="CK5" s="2" t="s">
+      <c r="CL5" s="2" t="s">
         <v>382</v>
       </c>
-      <c r="CL5" s="2" t="s">
+      <c r="CM5" s="2" t="s">
         <v>383</v>
       </c>
-      <c r="CM5" s="2" t="s">
+      <c r="CN5" s="2" t="s">
         <v>384</v>
       </c>
-      <c r="CN5" s="2" t="s">
+      <c r="CO5" s="2" t="s">
         <v>385</v>
       </c>
-      <c r="CO5" s="2" t="s">
+      <c r="CP5" s="2" t="s">
         <v>386</v>
       </c>
-      <c r="CP5" s="2" t="s">
+      <c r="CQ5" s="2" t="s">
         <v>387</v>
       </c>
-      <c r="CQ5" s="2" t="s">
+      <c r="CR5" s="2" t="s">
         <v>388</v>
       </c>
-      <c r="CR5" s="2" t="s">
+      <c r="CS5" s="2" t="s">
         <v>389</v>
-      </c>
-      <c r="CS5" s="2" t="s">
-        <v>390</v>
       </c>
     </row>
     <row r="6" spans="1:97" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>99</v>
+        <v>454</v>
       </c>
       <c r="B6" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="I6" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="J6" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="K6" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="L6" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="M6" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="N6" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="O6" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="P6" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="Q6" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="R6" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="C6" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="F6" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="G6" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="H6" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="I6" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="J6" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="K6" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="L6" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="M6" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="N6" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="O6" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="P6" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="Q6" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="R6" s="2" t="s">
+      <c r="S6" s="2" t="s">
+        <v>390</v>
+      </c>
+      <c r="T6" s="2" t="s">
+        <v>391</v>
+      </c>
+      <c r="U6" s="2" t="s">
+        <v>392</v>
+      </c>
+      <c r="V6" s="2" t="s">
+        <v>393</v>
+      </c>
+      <c r="W6" s="2" t="s">
+        <v>394</v>
+      </c>
+      <c r="X6" s="2" t="s">
+        <v>395</v>
+      </c>
+      <c r="Y6" s="2" t="s">
+        <v>396</v>
+      </c>
+      <c r="Z6" s="2" t="s">
+        <v>397</v>
+      </c>
+      <c r="AA6" s="2" t="s">
+        <v>398</v>
+      </c>
+      <c r="AB6" s="2" t="s">
+        <v>399</v>
+      </c>
+      <c r="AC6" s="2" t="s">
+        <v>400</v>
+      </c>
+      <c r="AD6" s="2" t="s">
+        <v>401</v>
+      </c>
+      <c r="AE6" s="2" t="s">
+        <v>402</v>
+      </c>
+      <c r="AF6" s="2" t="s">
+        <v>403</v>
+      </c>
+      <c r="AG6" s="2" t="s">
+        <v>404</v>
+      </c>
+      <c r="AH6" s="2" t="s">
+        <v>405</v>
+      </c>
+      <c r="AI6" s="2" t="s">
+        <v>406</v>
+      </c>
+      <c r="AJ6" s="2" t="s">
+        <v>407</v>
+      </c>
+      <c r="AK6" s="2" t="s">
+        <v>408</v>
+      </c>
+      <c r="AL6" s="2" t="s">
+        <v>409</v>
+      </c>
+      <c r="AM6" s="2" t="s">
+        <v>410</v>
+      </c>
+      <c r="AN6" s="2" t="s">
+        <v>411</v>
+      </c>
+      <c r="AO6" s="2" t="s">
+        <v>412</v>
+      </c>
+      <c r="AP6" s="2" t="s">
+        <v>413</v>
+      </c>
+      <c r="AQ6" s="2" t="s">
+        <v>414</v>
+      </c>
+      <c r="AR6" s="2" t="s">
+        <v>415</v>
+      </c>
+      <c r="AS6" s="2" t="s">
+        <v>416</v>
+      </c>
+      <c r="AT6" s="2" t="s">
+        <v>417</v>
+      </c>
+      <c r="AU6" s="2" t="s">
+        <v>418</v>
+      </c>
+      <c r="AV6" s="2" t="s">
+        <v>419</v>
+      </c>
+      <c r="AW6" s="2" t="s">
+        <v>420</v>
+      </c>
+      <c r="AX6" s="2" t="s">
+        <v>421</v>
+      </c>
+      <c r="AY6" s="2" t="s">
+        <v>422</v>
+      </c>
+      <c r="AZ6" s="2" t="s">
+        <v>423</v>
+      </c>
+      <c r="BA6" s="2" t="s">
+        <v>424</v>
+      </c>
+      <c r="BB6" s="2" t="s">
+        <v>425</v>
+      </c>
+      <c r="BC6" s="2" t="s">
+        <v>426</v>
+      </c>
+      <c r="BD6" s="2" t="s">
+        <v>427</v>
+      </c>
+      <c r="BE6" s="2" t="s">
+        <v>428</v>
+      </c>
+      <c r="BF6" s="2" t="s">
+        <v>429</v>
+      </c>
+      <c r="BG6" s="2" t="s">
+        <v>430</v>
+      </c>
+      <c r="BH6" s="2" t="s">
+        <v>431</v>
+      </c>
+      <c r="BI6" s="2" t="s">
+        <v>432</v>
+      </c>
+      <c r="BJ6" s="2" t="s">
+        <v>433</v>
+      </c>
+      <c r="BK6" s="2" t="s">
+        <v>434</v>
+      </c>
+      <c r="BL6" s="2" t="s">
+        <v>435</v>
+      </c>
+      <c r="BM6" s="2" t="s">
+        <v>436</v>
+      </c>
+      <c r="BN6" s="2" t="s">
+        <v>437</v>
+      </c>
+      <c r="BO6" s="2" t="s">
+        <v>438</v>
+      </c>
+      <c r="BP6" s="2" t="s">
+        <v>439</v>
+      </c>
+      <c r="BQ6" s="2" t="s">
+        <v>440</v>
+      </c>
+      <c r="BR6" s="2" t="s">
+        <v>441</v>
+      </c>
+      <c r="BS6" s="2" t="s">
+        <v>442</v>
+      </c>
+      <c r="BT6" s="2" t="s">
+        <v>443</v>
+      </c>
+      <c r="BU6" s="2" t="s">
+        <v>444</v>
+      </c>
+      <c r="BV6" s="2" t="s">
+        <v>445</v>
+      </c>
+      <c r="BW6" s="2" t="s">
+        <v>446</v>
+      </c>
+      <c r="BX6" s="2" t="s">
+        <v>447</v>
+      </c>
+      <c r="BY6" s="2" t="s">
+        <v>448</v>
+      </c>
+      <c r="BZ6" s="2" t="s">
+        <v>449</v>
+      </c>
+      <c r="CA6" s="2" t="s">
+        <v>450</v>
+      </c>
+      <c r="CB6" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="S6" s="2" t="s">
-        <v>391</v>
-      </c>
-      <c r="T6" s="2" t="s">
-        <v>392</v>
-      </c>
-      <c r="U6" s="2" t="s">
-        <v>393</v>
-      </c>
-      <c r="V6" s="2" t="s">
-        <v>394</v>
-      </c>
-      <c r="W6" s="2" t="s">
-        <v>395</v>
-      </c>
-      <c r="X6" s="2" t="s">
-        <v>396</v>
-      </c>
-      <c r="Y6" s="2" t="s">
-        <v>397</v>
-      </c>
-      <c r="Z6" s="2" t="s">
-        <v>398</v>
-      </c>
-      <c r="AA6" s="2" t="s">
-        <v>399</v>
-      </c>
-      <c r="AB6" s="2" t="s">
-        <v>400</v>
-      </c>
-      <c r="AC6" s="2" t="s">
-        <v>401</v>
-      </c>
-      <c r="AD6" s="2" t="s">
-        <v>402</v>
-      </c>
-      <c r="AE6" s="2" t="s">
-        <v>403</v>
-      </c>
-      <c r="AF6" s="2" t="s">
-        <v>404</v>
-      </c>
-      <c r="AG6" s="2" t="s">
-        <v>405</v>
-      </c>
-      <c r="AH6" s="2" t="s">
-        <v>406</v>
-      </c>
-      <c r="AI6" s="2" t="s">
-        <v>407</v>
-      </c>
-      <c r="AJ6" s="2" t="s">
-        <v>408</v>
-      </c>
-      <c r="AK6" s="2" t="s">
-        <v>409</v>
-      </c>
-      <c r="AL6" s="2" t="s">
-        <v>410</v>
-      </c>
-      <c r="AM6" s="2" t="s">
-        <v>411</v>
-      </c>
-      <c r="AN6" s="2" t="s">
-        <v>412</v>
-      </c>
-      <c r="AO6" s="2" t="s">
-        <v>413</v>
-      </c>
-      <c r="AP6" s="2" t="s">
-        <v>414</v>
-      </c>
-      <c r="AQ6" s="2" t="s">
-        <v>415</v>
-      </c>
-      <c r="AR6" s="2" t="s">
-        <v>416</v>
-      </c>
-      <c r="AS6" s="2" t="s">
-        <v>417</v>
-      </c>
-      <c r="AT6" s="2" t="s">
-        <v>418</v>
-      </c>
-      <c r="AU6" s="2" t="s">
-        <v>419</v>
-      </c>
-      <c r="AV6" s="2" t="s">
-        <v>420</v>
-      </c>
-      <c r="AW6" s="2" t="s">
-        <v>421</v>
-      </c>
-      <c r="AX6" s="2" t="s">
-        <v>422</v>
-      </c>
-      <c r="AY6" s="2" t="s">
-        <v>423</v>
-      </c>
-      <c r="AZ6" s="2" t="s">
-        <v>424</v>
-      </c>
-      <c r="BA6" s="2" t="s">
-        <v>425</v>
-      </c>
-      <c r="BB6" s="2" t="s">
-        <v>426</v>
-      </c>
-      <c r="BC6" s="2" t="s">
-        <v>427</v>
-      </c>
-      <c r="BD6" s="2" t="s">
-        <v>428</v>
-      </c>
-      <c r="BE6" s="2" t="s">
-        <v>429</v>
-      </c>
-      <c r="BF6" s="2" t="s">
-        <v>430</v>
-      </c>
-      <c r="BG6" s="2" t="s">
-        <v>431</v>
-      </c>
-      <c r="BH6" s="2" t="s">
-        <v>432</v>
-      </c>
-      <c r="BI6" s="2" t="s">
-        <v>433</v>
-      </c>
-      <c r="BJ6" s="2" t="s">
-        <v>434</v>
-      </c>
-      <c r="BK6" s="2" t="s">
-        <v>435</v>
-      </c>
-      <c r="BL6" s="2" t="s">
-        <v>436</v>
-      </c>
-      <c r="BM6" s="2" t="s">
-        <v>437</v>
-      </c>
-      <c r="BN6" s="2" t="s">
-        <v>438</v>
-      </c>
-      <c r="BO6" s="2" t="s">
-        <v>439</v>
-      </c>
-      <c r="BP6" s="2" t="s">
-        <v>440</v>
-      </c>
-      <c r="BQ6" s="2" t="s">
-        <v>441</v>
-      </c>
-      <c r="BR6" s="2" t="s">
-        <v>442</v>
-      </c>
-      <c r="BS6" s="2" t="s">
-        <v>443</v>
-      </c>
-      <c r="BT6" s="2" t="s">
-        <v>444</v>
-      </c>
-      <c r="BU6" s="2" t="s">
-        <v>445</v>
-      </c>
-      <c r="BV6" s="2" t="s">
-        <v>446</v>
-      </c>
-      <c r="BW6" s="2" t="s">
-        <v>447</v>
-      </c>
-      <c r="BX6" s="2" t="s">
-        <v>448</v>
-      </c>
-      <c r="BY6" s="2" t="s">
-        <v>449</v>
-      </c>
-      <c r="BZ6" s="2" t="s">
-        <v>450</v>
-      </c>
-      <c r="CA6" s="2" t="s">
-        <v>451</v>
-      </c>
-      <c r="CB6" s="2" t="s">
-        <v>110</v>
-      </c>
       <c r="CC6" s="2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="CD6" s="2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="CE6" s="2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="CF6" s="2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="CG6" s="2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="CH6" s="2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="CI6" s="2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="CJ6" s="2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="CK6" s="2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="CL6" s="2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="CM6" s="2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="CN6" s="2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="CO6" s="2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="CP6" s="2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="CQ6" s="2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="CR6" s="2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="CS6" s="2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="7" spans="1:97" x14ac:dyDescent="0.25">
@@ -8942,7 +8955,7 @@
     </row>
     <row r="8" spans="1:97" ht="27.6" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B8">
         <f>MAX(B7:CS7)+4000+4000</f>
@@ -9331,7 +9344,7 @@
     </row>
     <row r="9" spans="1:97" ht="27.6" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B9" s="5">
         <f>B7/B8</f>
@@ -9720,7 +9733,7 @@
     </row>
     <row r="10" spans="1:97" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B10">
         <f>B8*0.38</f>
@@ -9729,7 +9742,7 @@
     </row>
     <row r="11" spans="1:97" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B11">
         <f>MIN(B7:CS7)</f>
@@ -10333,7 +10346,7 @@
     </row>
     <row r="26" spans="1:97" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B26">
         <v>42377.79</v>
@@ -10626,7 +10639,7 @@
     </row>
     <row r="27" spans="1:97" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B27">
         <v>36714.320000000007</v>
@@ -10919,7 +10932,7 @@
     </row>
     <row r="28" spans="1:97" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B28">
         <v>36220.65</v>
@@ -11518,7 +11531,7 @@
     </row>
     <row r="2" spans="1:97" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B2">
         <v>24353.79</v>
@@ -12404,7 +12417,7 @@
     </row>
     <row r="2" spans="1:193" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B2">
         <v>43120.55</v>

</xml_diff>